<commit_message>
Pasta legislação com o texto das normas (Senado, Receita e Câmara) e CPP do Anexo IV com a divisão da folha
scripts/baixar_legislacao.py baixa leis (Normas.leg.br, compilação vigente), atos da Receita (visão multivigente), PDFs oficiais e
projetos da Câmara para legislação/ com índice. A leitura da IN RFB 2.110/2022 (arts. 168 a 171) substitui a estimativa da CPP fora do DAS
em atividades mistas: folha só do Anexo IV, só dos outros Anexos e concomitante. Premissas 82 e 83.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FVrp8HXiJ3fo8syeVkDidK
</commit_message>
<xml_diff>
--- a/kit-de-teste/6-casos-de-validacao.xlsx
+++ b/kit-de-teste/6-casos-de-validacao.xlsx
@@ -13371,7 +13371,7 @@
       </c>
       <c r="C394" s="6" t="inlineStr">
         <is>
-          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS estimada na proporção da receita do Anexo IV (regra de repartição da folha não lida: confirme); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
+          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS na proporção da receita do Anexo IV, com todos os empregados atuando nas duas atividades (IN RFB 2.110/2022, arts. 168 a 171); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
         </is>
       </c>
       <c r="D394" s="5" t="inlineStr">
@@ -13403,7 +13403,7 @@
       </c>
       <c r="C395" s="6" t="inlineStr">
         <is>
-          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS estimada na proporção da receita do Anexo IV (regra de repartição da folha não lida: confirme); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
+          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS na proporção da receita do Anexo IV, com todos os empregados atuando nas duas atividades (IN RFB 2.110/2022, arts. 168 a 171); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
         </is>
       </c>
       <c r="D395" s="5" t="inlineStr">
@@ -13435,7 +13435,7 @@
       </c>
       <c r="C396" s="10" t="inlineStr">
         <is>
-          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS estimada na proporção da receita do Anexo IV (regra de repartição da folha não lida: confirme); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
+          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS na proporção da receita do Anexo IV, com todos os empregados atuando nas duas atividades (IN RFB 2.110/2022, arts. 168 a 171); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
         </is>
       </c>
       <c r="D396" s="9" t="inlineStr">
@@ -13468,7 +13468,7 @@
       </c>
       <c r="C397" s="14" t="inlineStr">
         <is>
-          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS estimada na proporção da receita do Anexo IV (regra de repartição da folha não lida: confirme); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
+          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS na proporção da receita do Anexo IV, com todos os empregados atuando nas duas atividades (IN RFB 2.110/2022, arts. 168 a 171); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
         </is>
       </c>
       <c r="D397" s="13" t="inlineStr">
@@ -13500,7 +13500,7 @@
       </c>
       <c r="C398" s="14" t="inlineStr">
         <is>
-          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS estimada na proporção da receita do Anexo IV (regra de repartição da folha não lida: confirme); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
+          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS na proporção da receita do Anexo IV, com todos os empregados atuando nas duas atividades (IN RFB 2.110/2022, arts. 168 a 171); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
         </is>
       </c>
       <c r="D398" s="13" t="inlineStr">
@@ -13532,7 +13532,7 @@
       </c>
       <c r="C399" s="14" t="inlineStr">
         <is>
-          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS estimada na proporção da receita do Anexo IV (regra de repartição da folha não lida: confirme); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
+          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS na proporção da receita do Anexo IV, com todos os empregados atuando nas duas atividades (IN RFB 2.110/2022, arts. 168 a 171); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
         </is>
       </c>
       <c r="D399" s="13" t="inlineStr">
@@ -13564,7 +13564,7 @@
       </c>
       <c r="C400" s="14" t="inlineStr">
         <is>
-          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS estimada na proporção da receita do Anexo IV (regra de repartição da folha não lida: confirme); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
+          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS na proporção da receita do Anexo IV, com todos os empregados atuando nas duas atividades (IN RFB 2.110/2022, arts. 168 a 171); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
         </is>
       </c>
       <c r="D400" s="13" t="inlineStr">
@@ -13596,7 +13596,7 @@
       </c>
       <c r="C401" s="14" t="inlineStr">
         <is>
-          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS estimada na proporção da receita do Anexo IV (regra de repartição da folha não lida: confirme); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
+          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS na proporção da receita do Anexo IV, com todos os empregados atuando nas duas atividades (IN RFB 2.110/2022, arts. 168 a 171); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
         </is>
       </c>
       <c r="D401" s="13" t="inlineStr">
@@ -13628,7 +13628,7 @@
       </c>
       <c r="C402" s="14" t="inlineStr">
         <is>
-          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS estimada na proporção da receita do Anexo IV (regra de repartição da folha não lida: confirme); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
+          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS na proporção da receita do Anexo IV, com todos os empregados atuando nas duas atividades (IN RFB 2.110/2022, arts. 168 a 171); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
         </is>
       </c>
       <c r="D402" s="13" t="inlineStr">
@@ -13660,7 +13660,7 @@
       </c>
       <c r="C403" s="14" t="inlineStr">
         <is>
-          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS estimada na proporção da receita do Anexo IV (regra de repartição da folha não lida: confirme); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
+          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS na proporção da receita do Anexo IV, com todos os empregados atuando nas duas atividades (IN RFB 2.110/2022, arts. 168 a 171); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
         </is>
       </c>
       <c r="D403" s="13" t="inlineStr">
@@ -13692,7 +13692,7 @@
       </c>
       <c r="C404" s="17" t="inlineStr">
         <is>
-          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS estimada na proporção da receita do Anexo IV (regra de repartição da folha não lida: confirme); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
+          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS na proporção da receita do Anexo IV, com todos os empregados atuando nas duas atividades (IN RFB 2.110/2022, arts. 168 a 171); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
         </is>
       </c>
       <c r="D404" s="16" t="inlineStr">
@@ -13725,7 +13725,7 @@
       </c>
       <c r="C405" s="6" t="inlineStr">
         <is>
-          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS estimada na proporção da receita do Anexo IV (regra de repartição da folha não lida: confirme); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
+          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS na proporção da receita do Anexo IV, com todos os empregados atuando nas duas atividades (IN RFB 2.110/2022, arts. 168 a 171); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
         </is>
       </c>
       <c r="D405" s="5" t="inlineStr">
@@ -13757,7 +13757,7 @@
       </c>
       <c r="C406" s="6" t="inlineStr">
         <is>
-          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS estimada na proporção da receita do Anexo IV (regra de repartição da folha não lida: confirme); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
+          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS na proporção da receita do Anexo IV, com todos os empregados atuando nas duas atividades (IN RFB 2.110/2022, arts. 168 a 171); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
         </is>
       </c>
       <c r="D406" s="5" t="inlineStr">
@@ -13789,7 +13789,7 @@
       </c>
       <c r="C407" s="6" t="inlineStr">
         <is>
-          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS estimada na proporção da receita do Anexo IV (regra de repartição da folha não lida: confirme); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
+          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS na proporção da receita do Anexo IV, com todos os empregados atuando nas duas atividades (IN RFB 2.110/2022, arts. 168 a 171); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
         </is>
       </c>
       <c r="D407" s="5" t="inlineStr">
@@ -13821,7 +13821,7 @@
       </c>
       <c r="C408" s="6" t="inlineStr">
         <is>
-          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS estimada na proporção da receita do Anexo IV (regra de repartição da folha não lida: confirme); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
+          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS na proporção da receita do Anexo IV, com todos os empregados atuando nas duas atividades (IN RFB 2.110/2022, arts. 168 a 171); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
         </is>
       </c>
       <c r="D408" s="5" t="inlineStr">
@@ -13853,7 +13853,7 @@
       </c>
       <c r="C409" s="6" t="inlineStr">
         <is>
-          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS estimada na proporção da receita do Anexo IV (regra de repartição da folha não lida: confirme); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
+          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS na proporção da receita do Anexo IV, com todos os empregados atuando nas duas atividades (IN RFB 2.110/2022, arts. 168 a 171); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
         </is>
       </c>
       <c r="D409" s="5" t="inlineStr">
@@ -13885,7 +13885,7 @@
       </c>
       <c r="C410" s="6" t="inlineStr">
         <is>
-          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS estimada na proporção da receita do Anexo IV (regra de repartição da folha não lida: confirme); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
+          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS na proporção da receita do Anexo IV, com todos os empregados atuando nas duas atividades (IN RFB 2.110/2022, arts. 168 a 171); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
         </is>
       </c>
       <c r="D410" s="5" t="inlineStr">
@@ -13917,7 +13917,7 @@
       </c>
       <c r="C411" s="6" t="inlineStr">
         <is>
-          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS estimada na proporção da receita do Anexo IV (regra de repartição da folha não lida: confirme); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
+          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS na proporção da receita do Anexo IV, com todos os empregados atuando nas duas atividades (IN RFB 2.110/2022, arts. 168 a 171); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
         </is>
       </c>
       <c r="D411" s="5" t="inlineStr">
@@ -13949,7 +13949,7 @@
       </c>
       <c r="C412" s="10" t="inlineStr">
         <is>
-          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS estimada na proporção da receita do Anexo IV (regra de repartição da folha não lida: confirme); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
+          <t>Advocacia (Anexo IV, R$ 600 mil) + comércio (R$ 300 mil): CPP fora do DAS na proporção da receita do Anexo IV, com todos os empregados atuando nas duas atividades (IN RFB 2.110/2022, arts. 168 a 171); servico_anexo_iv; receita R$ 900.000,00/ano; folha CLT R$ 120.000,00; pró-labore R$ 36.000,00; compras R$ 150.000,00; ano 2026; receita em comercio R$ 300.000,00; ISS 5%</t>
         </is>
       </c>
       <c r="D412" s="9" t="inlineStr">
@@ -21105,7 +21105,7 @@
       </c>
       <c r="E150" s="6" t="inlineStr">
         <is>
-          <t>LC 123/2006, art. 18, §5º-C e art. 13, VI</t>
+          <t>LC 123/2006, art. 18, § 5º-C e art. 13, VI</t>
         </is>
       </c>
     </row>
@@ -29887,7 +29887,7 @@
       </c>
       <c r="E504" s="6" t="inlineStr">
         <is>
-          <t>LC 123/2006, art. 18, §5º-C e art. 13, VI</t>
+          <t>LC 123/2006, art. 18, § 5º-C e art. 13, VI</t>
         </is>
       </c>
     </row>
@@ -37213,7 +37213,7 @@
       </c>
       <c r="C798" s="6" t="inlineStr">
         <is>
-          <t>(R$ 120.000,00 x (20,00% + 2,00% RAT) + R$ 36.000,00 x 20,00%) x 66,67% da receita no Anexo IV</t>
+          <t>(R$ 120.000,00 x (20,00% + 2,00% RAT) + R$ 36.000,00 x 20,00%) x (0% da folha só do Anexo IV + 100% nas duas atividades x 66,67% da receita no Anexo IV) = x 66,67%</t>
         </is>
       </c>
       <c r="D798" s="7" t="n">
@@ -37221,7 +37221,7 @@
       </c>
       <c r="E798" s="6" t="inlineStr">
         <is>
-          <t>LC 123/2006, art. 18, §5º-C e art. 13, VI</t>
+          <t>LC 123/2006, art. 18, § 5º-C e art. 13, VI; Res. CGSN 140/2018, art. 147; IN RFB 2.110/2022, arts. 168 a 171</t>
         </is>
       </c>
     </row>
@@ -45824,7 +45824,7 @@
       </c>
       <c r="B108" s="6" t="inlineStr">
         <is>
-          <t>Atividade do Anexo IV junto com outras: a CPP patronal sai do DAS só na atividade do Anexo IV, mas o texto que reparte a folha entre as atividades não foi lido (portais oficiais indisponíveis em 27/10/2026). O Tolaris estima a CPP fora do DAS na proporção da receita do Anexo IV. Confirme com o contador como a folha é apropriada.</t>
+          <t>Atividade do Anexo IV junto com outras: a CPP patronal sai do DAS só para a folha ligada ao Anexo IV (IN RFB 2.110/2022, arts. 168 a 171): empregados só do Anexo IV pagam a CPP inteira, os que atuam nas duas atividades pagam na proporção da receita do Anexo IV e os que atuam só nas outras já estão cobertos pelo DAS. Sem a divisão da folha por atividade, o Tolaris tratou todos os empregados como atuando nas duas atividades (CPP na proporção da receita do Anexo IV).</t>
         </is>
       </c>
     </row>

</xml_diff>